<commit_message>
fix: sua header Excel dung dinh dang tieng Viet co dau
</commit_message>
<xml_diff>
--- a/Danh_Sach_Khach_Hang.xlsx
+++ b/Danh_Sach_Khach_Hang.xlsx
@@ -450,12 +450,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>So dien thoai</t>
+          <t>Số điện thoại</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ho ten</t>
+          <t>Họ tên</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Nguon</t>
+          <t>Nguồn</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Khach hang 1</t>
+          <t>Khách hàng 1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>

</xml_diff>